<commit_message>
chore: sync Stata-Tools releases and regenerated demos
Publish gcomp 2.0.0 and iivw 4.0.0, syncing their .ado, .pkg,
.sthlp, and README metadata. Regenerate datamap 1.6.7 demo datasets
and outputs, including decimal formatting and privacy console capture.
Simplify diagtab's check_xlsx.py and refresh demo_diagtab.xlsx. Correct
the package catalog to list tabtools 2.0.0 instead of 2.1.0.
</commit_message>
<xml_diff>
--- a/tabtools/demo/demo_table1.xlsx
+++ b/tabtools/demo/demo_table1.xlsx
@@ -14,9 +14,9 @@
     <sheet name="Table 1 Formats" sheetId="6" r:id="rId8"/>
     <sheet name="Table 1 Missing" sheetId="7" r:id="rId9"/>
     <sheet name="Table 1 Custom" sheetId="8" r:id="rId10"/>
-    <sheet name="Table 1 NEJM" sheetId="9" r:id="rId11"/>
-    <sheet name="Theme BMJ" sheetId="10" r:id="rId12"/>
-    <sheet name="Theme APA" sheetId="11" r:id="rId13"/>
+    <sheet name="Table 1 Compact" sheetId="9" r:id="rId11"/>
+    <sheet name="Explicit Arial" sheetId="10" r:id="rId12"/>
+    <sheet name="Explicit Serif" sheetId="11" r:id="rId13"/>
     <sheet name="Small Cells Primary" sheetId="12" r:id="rId14"/>
     <sheet name="Small Cells Complement" sheetId="13" r:id="rId15"/>
     <sheet name="Small Cells Binary" sheetId="14" r:id="rId16"/>
@@ -763,13 +763,13 @@
     <t>SD shown as mean [SD]. IQR uses 'to' separator. Row % for categoricals.</t>
   </si>
   <si>
-    <t>Table 1. Baseline Characteristics (NEJM Style)</t>
-  </si>
-  <si>
-    <t>Table 1. Baseline Characteristics (BMJ Style)</t>
-  </si>
-  <si>
-    <t>Table 1. Baseline Characteristics (APA Style)</t>
+    <t>Table 1. Baseline Characteristics (Compact Style)</t>
+  </si>
+  <si>
+    <t>Table 1. Baseline Characteristics (Arial Style)</t>
+  </si>
+  <si>
+    <t>Table 1. Baseline Characteristics (Serif Style)</t>
   </si>
   <si>
     <t>Small-cell suppression: primary counts only</t>

</xml_diff>